<commit_message>
Normalize punctuation in sample data
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -532,7 +532,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 · 앱 기본 더미 식비와 동일 · 특이 사항/배분 제외 사례 없음</x:v>
+        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 앱 기본 더미 식비와 동일 , 특이 사항/배분 제외 사례 없음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -768,7 +768,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 · 앱 기본 더미 식비와 동일 · 특이 사항/배분 제외 사례 없음</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 앱 기본 더미 식비와 동일 , 특이 사항/배분 제외 사례 없음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>

</xml_diff>

<commit_message>
Gate meal allocation by approval status
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Rf267a855b1394234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="Rea6bde29bd0341c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="R66b5b294035c4c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R0b7446a09a8d49b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="#,##0&quot;원&quot;"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -50,6 +51,11 @@
       <x:sz val="10"/>
       <x:color rgb="FF1D252C"/>
       <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D252C"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="6">
@@ -126,7 +132,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -220,18 +226,111 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="200" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="10">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FFBF4B4B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -241,7 +340,7 @@
         <x:color rgb="FF28785F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -252,7 +351,7 @@
         <x:color rgb="FFBF4B4B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -262,8 +361,68 @@
         <x:color rgb="FF28785F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF28785F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFBF4B4B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF1F4E78"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF28785F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFBF4B4B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF1F4E78"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -272,8 +431,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SamildolMealsTable" displayName="SamildolMealsTable" ref="A5:J9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:J9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SamildolMealsTable" displayName="SamildolMealsTable" ref="A5:J13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J13"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="날짜"/>
     <x:tableColumn id="2" name="결제 시간"/>
@@ -291,8 +450,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SamdeheonMealsTable" displayName="SamdeheonMealsTable" ref="A5:J9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:J9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SamdeheonMealsTable" displayName="SamdeheonMealsTable" ref="A5:J13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J13"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="날짜"/>
     <x:tableColumn id="2" name="결제 시간"/>
@@ -532,7 +691,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 앱 기본 더미 식비와 동일 , 특이 사항/배분 제외 사례 없음</x:v>
+        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 파일 전용 추가 식사 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -720,6 +879,141 @@
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="72" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B10" s="73" t="str">
+        <x:v>18:30</x:v>
+      </x:c>
+      <x:c r="C10" s="65" t="str">
+        <x:v>팬미팅 연습 저녁</x:v>
+      </x:c>
+      <x:c r="D10" s="80" t="n">
+        <x:v>145000</x:v>
+      </x:c>
+      <x:c r="E10" s="65" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F10" s="73" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G10" s="76" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H10" s="77" t="n">
+        <x:f>ROUND(D10/G10,0)</x:f>
+        <x:v>29000</x:v>
+      </x:c>
+      <x:c r="I10" s="73" t="str">
+        <x:f>IF(H10&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J10" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="72" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B11" s="73" t="str">
+        <x:v>12:10</x:v>
+      </x:c>
+      <x:c r="C11" s="65" t="str">
+        <x:v>콘텐츠 촬영 도시락</x:v>
+      </x:c>
+      <x:c r="D11" s="80" t="n">
+        <x:v>162000</x:v>
+      </x:c>
+      <x:c r="E11" s="65" t="str">
+        <x:v>Haru, Seo, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F11" s="73" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G11" s="76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H11" s="77" t="n">
+        <x:f>ROUND(D11/G11,0)</x:f>
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="I11" s="73" t="str">
+        <x:v>승인 완료</x:v>
+      </x:c>
+      <x:c r="J11" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="72" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B12" s="73" t="str">
+        <x:v>13:00</x:v>
+      </x:c>
+      <x:c r="C12" s="65" t="str">
+        <x:v>월간회의 점심</x:v>
+      </x:c>
+      <x:c r="D12" s="80" t="n">
+        <x:v>138000</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F12" s="73" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G12" s="76" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H12" s="77" t="n">
+        <x:f>ROUND(D12/G12,0)</x:f>
+        <x:v>27600</x:v>
+      </x:c>
+      <x:c r="I12" s="73" t="str">
+        <x:f>IF(H12&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J12" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="74" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>18:20</x:v>
+      </x:c>
+      <x:c r="C13" s="69" t="str">
+        <x:v>마감 리허설 저녁</x:v>
+      </x:c>
+      <x:c r="D13" s="81" t="n">
+        <x:v>175000</x:v>
+      </x:c>
+      <x:c r="E13" s="69" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F13" s="75" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G13" s="78" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H13" s="79" t="n">
+        <x:f>ROUND(D13/G13,0)</x:f>
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="I13" s="75" t="str">
+        <x:f>IF(H13&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J13" s="75" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -729,9 +1023,14 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="승인 대기"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="자동 처리"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I10:I13">
+    <x:cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="자동 처리"/>
+    <x:cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="승인 대기"/>
+    <x:cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="승인 완료"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R557ec0110ab94021"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaedee2ff1284178"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -768,7 +1067,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 앱 기본 더미 식비와 동일 , 특이 사항/배분 제외 사례 없음</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 파일 전용 추가 식사 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -956,6 +1255,141 @@
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="72" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+      <x:c r="B10" s="73" t="str">
+        <x:v>12:05</x:v>
+      </x:c>
+      <x:c r="C10" s="65" t="str">
+        <x:v>녹음실 점심</x:v>
+      </x:c>
+      <x:c r="D10" s="80" t="n">
+        <x:v>112000</x:v>
+      </x:c>
+      <x:c r="E10" s="65" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F10" s="73" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G10" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H10" s="77" t="n">
+        <x:f>ROUND(D10/G10,0)</x:f>
+        <x:v>28000</x:v>
+      </x:c>
+      <x:c r="I10" s="73" t="str">
+        <x:f>IF(H10&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J10" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="72" t="n">
+        <x:v>46230</x:v>
+      </x:c>
+      <x:c r="B11" s="73" t="str">
+        <x:v>18:30</x:v>
+      </x:c>
+      <x:c r="C11" s="65" t="str">
+        <x:v>안무 연습 저녁</x:v>
+      </x:c>
+      <x:c r="D11" s="80" t="n">
+        <x:v>148000</x:v>
+      </x:c>
+      <x:c r="E11" s="65" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F11" s="73" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G11" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H11" s="77" t="n">
+        <x:f>ROUND(D11/G11,0)</x:f>
+        <x:v>37000</x:v>
+      </x:c>
+      <x:c r="I11" s="73" t="str">
+        <x:v>승인 완료</x:v>
+      </x:c>
+      <x:c r="J11" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="72" t="n">
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="B12" s="73" t="str">
+        <x:v>11:55</x:v>
+      </x:c>
+      <x:c r="C12" s="65" t="str">
+        <x:v>방송 리허설 도시락</x:v>
+      </x:c>
+      <x:c r="D12" s="80" t="n">
+        <x:v>124000</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F12" s="73" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G12" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H12" s="77" t="n">
+        <x:f>ROUND(D12/G12,0)</x:f>
+        <x:v>31000</x:v>
+      </x:c>
+      <x:c r="I12" s="73" t="str">
+        <x:f>IF(H12&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J12" s="73" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="74" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>19:10</x:v>
+      </x:c>
+      <x:c r="C13" s="69" t="str">
+        <x:v>월말 합주 저녁</x:v>
+      </x:c>
+      <x:c r="D13" s="81" t="n">
+        <x:v>108000</x:v>
+      </x:c>
+      <x:c r="E13" s="69" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F13" s="75" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G13" s="78" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H13" s="79" t="n">
+        <x:f>ROUND(D13/G13,0)</x:f>
+        <x:v>27000</x:v>
+      </x:c>
+      <x:c r="I13" s="75" t="str">
+        <x:f>IF(H13&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J13" s="75" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -965,9 +1399,14 @@
     <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="승인 대기"/>
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="자동 처리"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I10:I13">
+    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="자동 처리"/>
+    <x:cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="승인 대기"/>
+    <x:cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="승인 완료"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc24aa87173344835"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7623986506b4650"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add same-hour approval sample meals
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="R66b5b294035c4c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R0b7446a09a8d49b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Rba7646f9d0244f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R97469dbee388451f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -57,8 +57,19 @@
       <x:color rgb="FF1D252C"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFE26B5B"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,8 +96,28 @@
         <x:fgColor rgb="FF1F7A8C"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC7E8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -128,11 +159,25 @@
         <x:color rgb="FFDFE6EA"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE0A458"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE0A458"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE0A458"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE0A458"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -318,6 +363,60 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="201" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="200" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1030,7 +1129,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaedee2ff1284178"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64503fd56dcb41f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1067,7 +1166,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 파일 전용 추가 식사 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 동일 시간대 3건 승인 확인용 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1087,6 +1186,14 @@
         <x:v>30000</x:v>
       </x:c>
     </x:row>
+    <x:row r="4">
+      <x:c r="I4" s="85" t="str">
+        <x:v>동시간대 승인 기준</x:v>
+      </x:c>
+      <x:c r="J4" s="85" t="str">
+        <x:v>3건</x:v>
+      </x:c>
+    </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="18" t="str">
         <x:v>날짜</x:v>
@@ -1282,8 +1389,7 @@
         <x:v>28000</x:v>
       </x:c>
       <x:c r="I10" s="73" t="str">
-        <x:f>IF(H10&gt;$J$3,"승인 대기","자동 처리")</x:f>
-        <x:v>자동 처리</x:v>
+        <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J10" s="73" t="str">
         <x:v>인사 마스터</x:v>
@@ -1387,6 +1493,70 @@
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J13" s="75" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="90" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+      <x:c r="B14" s="92" t="str">
+        <x:v>12:30</x:v>
+      </x:c>
+      <x:c r="C14" s="86" t="str">
+        <x:v>녹음실 추가 음료</x:v>
+      </x:c>
+      <x:c r="D14" s="96" t="n">
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="E14" s="86" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F14" s="92" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G14" s="100" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H14" s="102" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I14" s="108" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J14" s="92" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="91" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>12:50</x:v>
+      </x:c>
+      <x:c r="C15" s="87" t="str">
+        <x:v>녹음실 간식 결제</x:v>
+      </x:c>
+      <x:c r="D15" s="97" t="n">
+        <x:v>36000</x:v>
+      </x:c>
+      <x:c r="E15" s="87" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G15" s="101" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H15" s="103" t="n">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="I15" s="109" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J15" s="93" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1406,7 +1576,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7623986506b4650"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeeb7f4a238149f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Link meal allocation to activity records
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Rba7646f9d0244f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R97469dbee388451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Re5f6ac442a07480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R473605a2fa6d43d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1129,7 +1129,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64503fd56dcb41f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112d1a21b2b44dc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1308,20 +1308,18 @@
         <x:v>54000</x:v>
       </x:c>
       <x:c r="E8" s="39" t="str">
-        <x:v>장현우, 김진현, Manager Choi</x:v>
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
       <x:c r="F8" s="39" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
       <x:c r="G8" s="27" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H8" s="36" t="n">
-        <x:f>ROUND(D8/G8,0)</x:f>
-        <x:v>27000</x:v>
+        <x:v>13500</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:f>IF(H8&gt;$J$3,"승인 대기","자동 처리")</x:f>
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J8" s="27" t="str">
@@ -1576,7 +1574,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeeb7f4a238149f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0069f869492a4192"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Align attendance samples with current meal dates
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Re5f6ac442a07480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R473605a2fa6d43d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Re1763d90d2df4a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R7a84932faa2c491e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +109,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFC7E8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -177,7 +187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="110">
+  <x:cellXfs count="114">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -417,6 +427,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1129,7 +1151,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112d1a21b2b44dc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94eed0a7b1964339"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1166,7 +1188,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-31 , 동일 시간대 3건 승인 확인용 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-22 , 2026-07-21 동일 시간대 3건 승인 확인용 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1249,11 +1271,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H6" s="35" t="n">
-        <x:f>ROUND(D6/G6,0)</x:f>
         <x:v>29500</x:v>
       </x:c>
-      <x:c r="I6" s="26" t="str">
-        <x:f>IF(H6&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I6" s="110" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J6" s="26" t="str">
@@ -1283,11 +1303,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H7" s="36" t="n">
-        <x:f>ROUND(D7/G7,0)</x:f>
         <x:v>33000</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
-        <x:f>IF(H7&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I7" s="111" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J7" s="27" t="str">
@@ -1299,7 +1317,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="B8" s="27" t="str">
-        <x:v>18:10</x:v>
+        <x:v>12:05</x:v>
       </x:c>
       <x:c r="C8" s="24" t="str">
         <x:v>라디오 대기 식사</x:v>
@@ -1319,8 +1337,8 @@
       <x:c r="H8" s="36" t="n">
         <x:v>13500</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
-        <x:v>자동 처리</x:v>
+      <x:c r="I8" s="111" t="str">
+        <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J8" s="27" t="str">
         <x:v>인사 마스터</x:v>
@@ -1328,16 +1346,16 @@
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
       <x:c r="A9" s="31" t="n">
-        <x:v>46228</x:v>
+        <x:v>46224</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>19:05</x:v>
+        <x:v>12:30</x:v>
       </x:c>
       <x:c r="C9" s="25" t="str">
-        <x:v>팬미팅 리허설 저녁</x:v>
+        <x:v>라디오 추가 음료</x:v>
       </x:c>
       <x:c r="D9" s="34" t="n">
-        <x:v>126000</x:v>
+        <x:v>24000</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
@@ -1349,11 +1367,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H9" s="37" t="n">
-        <x:f>ROUND(D9/G9,0)</x:f>
-        <x:v>31500</x:v>
-      </x:c>
-      <x:c r="I9" s="28" t="str">
-        <x:f>IF(H9&gt;$J$3,"승인 대기","자동 처리")</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I9" s="112" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J9" s="28" t="str">
@@ -1362,16 +1378,16 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="72" t="n">
-        <x:v>46229</x:v>
+        <x:v>46224</x:v>
       </x:c>
       <x:c r="B10" s="73" t="str">
-        <x:v>12:05</x:v>
+        <x:v>12:50</x:v>
       </x:c>
       <x:c r="C10" s="65" t="str">
-        <x:v>녹음실 점심</x:v>
+        <x:v>라디오 간식 결제</x:v>
       </x:c>
       <x:c r="D10" s="80" t="n">
-        <x:v>112000</x:v>
+        <x:v>36000</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
@@ -1383,10 +1399,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H10" s="77" t="n">
-        <x:f>ROUND(D10/G10,0)</x:f>
-        <x:v>28000</x:v>
-      </x:c>
-      <x:c r="I10" s="73" t="str">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="I10" s="113" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J10" s="73" t="str">
@@ -1394,169 +1409,64 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="72" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="B11" s="73" t="str">
-        <x:v>18:30</x:v>
-      </x:c>
-      <x:c r="C11" s="65" t="str">
-        <x:v>안무 연습 저녁</x:v>
-      </x:c>
-      <x:c r="D11" s="80" t="n">
-        <x:v>148000</x:v>
-      </x:c>
-      <x:c r="E11" s="65" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F11" s="73" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G11" s="76" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H11" s="77" t="n">
-        <x:f>ROUND(D11/G11,0)</x:f>
-        <x:v>37000</x:v>
-      </x:c>
-      <x:c r="I11" s="73" t="str">
-        <x:v>승인 완료</x:v>
-      </x:c>
-      <x:c r="J11" s="73" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
+      <x:c r="A11" s="72"/>
+      <x:c r="B11" s="73"/>
+      <x:c r="C11" s="65"/>
+      <x:c r="D11" s="80"/>
+      <x:c r="E11" s="65"/>
+      <x:c r="F11" s="73"/>
+      <x:c r="G11" s="76"/>
+      <x:c r="H11" s="77"/>
+      <x:c r="I11" s="73"/>
+      <x:c r="J11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="72" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="B12" s="73" t="str">
-        <x:v>11:55</x:v>
-      </x:c>
-      <x:c r="C12" s="65" t="str">
-        <x:v>방송 리허설 도시락</x:v>
-      </x:c>
-      <x:c r="D12" s="80" t="n">
-        <x:v>124000</x:v>
-      </x:c>
-      <x:c r="E12" s="65" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F12" s="73" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G12" s="76" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H12" s="77" t="n">
-        <x:f>ROUND(D12/G12,0)</x:f>
-        <x:v>31000</x:v>
-      </x:c>
-      <x:c r="I12" s="73" t="str">
-        <x:f>IF(H12&gt;$J$3,"승인 대기","자동 처리")</x:f>
-        <x:v>승인 대기</x:v>
-      </x:c>
-      <x:c r="J12" s="73" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
+      <x:c r="A12" s="72"/>
+      <x:c r="B12" s="73"/>
+      <x:c r="C12" s="65"/>
+      <x:c r="D12" s="80"/>
+      <x:c r="E12" s="65"/>
+      <x:c r="F12" s="73"/>
+      <x:c r="G12" s="76"/>
+      <x:c r="H12" s="77"/>
+      <x:c r="I12" s="73"/>
+      <x:c r="J12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="74" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="B13" s="75" t="str">
-        <x:v>19:10</x:v>
-      </x:c>
-      <x:c r="C13" s="69" t="str">
-        <x:v>월말 합주 저녁</x:v>
-      </x:c>
-      <x:c r="D13" s="81" t="n">
-        <x:v>108000</x:v>
-      </x:c>
-      <x:c r="E13" s="69" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F13" s="75" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G13" s="78" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H13" s="79" t="n">
-        <x:f>ROUND(D13/G13,0)</x:f>
-        <x:v>27000</x:v>
-      </x:c>
-      <x:c r="I13" s="75" t="str">
-        <x:f>IF(H13&gt;$J$3,"승인 대기","자동 처리")</x:f>
-        <x:v>자동 처리</x:v>
-      </x:c>
-      <x:c r="J13" s="75" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
+      <x:c r="A13" s="74"/>
+      <x:c r="B13" s="75"/>
+      <x:c r="C13" s="69"/>
+      <x:c r="D13" s="81"/>
+      <x:c r="E13" s="69"/>
+      <x:c r="F13" s="75"/>
+      <x:c r="G13" s="78"/>
+      <x:c r="H13" s="79"/>
+      <x:c r="I13" s="75"/>
+      <x:c r="J13" s="75"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="90" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B14" s="92" t="str">
-        <x:v>12:30</x:v>
-      </x:c>
-      <x:c r="C14" s="86" t="str">
-        <x:v>녹음실 추가 음료</x:v>
-      </x:c>
-      <x:c r="D14" s="96" t="n">
-        <x:v>24000</x:v>
-      </x:c>
-      <x:c r="E14" s="86" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F14" s="92" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G14" s="100" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H14" s="102" t="n">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="I14" s="108" t="str">
-        <x:v>승인 대기</x:v>
-      </x:c>
-      <x:c r="J14" s="92" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
+      <x:c r="A14" s="90"/>
+      <x:c r="B14" s="92"/>
+      <x:c r="C14" s="86"/>
+      <x:c r="D14" s="96"/>
+      <x:c r="E14" s="86"/>
+      <x:c r="F14" s="92"/>
+      <x:c r="G14" s="100"/>
+      <x:c r="H14" s="102"/>
+      <x:c r="I14" s="108"/>
+      <x:c r="J14" s="92"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="91" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="B15" s="93" t="str">
-        <x:v>12:50</x:v>
-      </x:c>
-      <x:c r="C15" s="87" t="str">
-        <x:v>녹음실 간식 결제</x:v>
-      </x:c>
-      <x:c r="D15" s="97" t="n">
-        <x:v>36000</x:v>
-      </x:c>
-      <x:c r="E15" s="87" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F15" s="93" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G15" s="101" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H15" s="103" t="n">
-        <x:v>9000</x:v>
-      </x:c>
-      <x:c r="I15" s="109" t="str">
-        <x:v>승인 대기</x:v>
-      </x:c>
-      <x:c r="J15" s="93" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
+      <x:c r="A15" s="91"/>
+      <x:c r="B15" s="93"/>
+      <x:c r="C15" s="87"/>
+      <x:c r="D15" s="97"/>
+      <x:c r="E15" s="87"/>
+      <x:c r="F15" s="93"/>
+      <x:c r="G15" s="101"/>
+      <x:c r="H15" s="103"/>
+      <x:c r="I15" s="109"/>
+      <x:c r="J15" s="93"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1574,7 +1484,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0069f869492a4192"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd91234efe092456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Build weekday-linked sample records
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Re1763d90d2df4a92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R7a84932faa2c491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="R17a40d1aa3f642f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R088776835ee740ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,6 +114,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -187,7 +202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="114">
+  <x:cellXfs count="119">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +455,11 @@
     <x:xf numFmtId="0" fontId="6" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -812,7 +832,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 파일 전용 추가 식사 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
+        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 주 5일 평일 출퇴근 기록과 일정표에 연동 , 앱 기본 식비에 자동 반영되지 않음</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -865,273 +885,354 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="29" t="n">
+      <x:c r="A6" s="115" t="n">
         <x:v>46204</x:v>
       </x:c>
-      <x:c r="B6" s="26" t="str">
+      <x:c r="B6" s="114" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C6" s="23" t="str">
+      <x:c r="C6" s="114" t="str">
         <x:v>배민 연습실 식사</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="n">
+      <x:c r="D6" s="116" t="n">
         <x:v>92000</x:v>
       </x:c>
-      <x:c r="E6" s="38" t="str">
+      <x:c r="E6" s="114" t="str">
         <x:v>Haru, Min, Seo, Lia, Manager Park</x:v>
       </x:c>
-      <x:c r="F6" s="38" t="str">
+      <x:c r="F6" s="114" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G6" s="26" t="n">
+      <x:c r="G6" s="114" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="35" t="n">
-        <x:f>ROUND(D6/G6,0)</x:f>
+      <x:c r="H6" s="116" t="n">
         <x:v>23000</x:v>
       </x:c>
-      <x:c r="I6" s="26" t="str">
-        <x:f>IF(H6&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I6" s="117" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J6" s="26" t="str">
+      <x:c r="J6" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
-      <x:c r="A7" s="30" t="n">
+      <x:c r="A7" s="44" t="n">
+        <x:v>46205</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>12:20</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>쇼케이스 준비 점심</x:v>
+      </x:c>
+      <x:c r="D7" s="46" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F7" s="45" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H7" s="46" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="I7" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="32" customHeight="1">
+      <x:c r="A8" s="115" t="n">
         <x:v>46206</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B8" s="114" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="str">
+      <x:c r="C8" s="114" t="str">
         <x:v>음악방송 도시락</x:v>
       </x:c>
-      <x:c r="D7" s="33" t="n">
+      <x:c r="D8" s="116" t="n">
         <x:v>165000</x:v>
       </x:c>
-      <x:c r="E7" s="39" t="str">
+      <x:c r="E8" s="114" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F7" s="39" t="str">
+      <x:c r="F8" s="114" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G7" s="27" t="n">
+      <x:c r="G8" s="114" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H7" s="36" t="n">
-        <x:f>ROUND(D7/G7,0)</x:f>
+      <x:c r="H8" s="116" t="n">
         <x:v>33000</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
-        <x:f>IF(H7&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I8" s="118" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J7" s="27" t="str">
+      <x:c r="J8" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="30" t="n">
+    <x:row r="9" ht="32" customHeight="1">
+      <x:c r="A9" s="44" t="n">
         <x:v>46209</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B9" s="45" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C8" s="24" t="str">
+      <x:c r="C9" s="45" t="str">
         <x:v>라디오 대기 간식</x:v>
       </x:c>
-      <x:c r="D8" s="33" t="n">
+      <x:c r="D9" s="46" t="n">
         <x:v>48000</x:v>
       </x:c>
-      <x:c r="E8" s="39" t="str">
+      <x:c r="E9" s="45" t="str">
         <x:v>Min, Seo, Manager Park</x:v>
       </x:c>
-      <x:c r="F8" s="39" t="str">
+      <x:c r="F9" s="45" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="n">
+      <x:c r="G9" s="45" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H8" s="36" t="n">
-        <x:f>ROUND(D8/G8,0)</x:f>
+      <x:c r="H9" s="46" t="n">
         <x:v>24000</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
-        <x:f>IF(H8&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I9" s="117" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J8" s="27" t="str">
+      <x:c r="J9" s="45" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
-      <x:c r="A9" s="31" t="n">
+    <x:row r="10">
+      <x:c r="A10" s="115" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="B10" s="114" t="str">
+        <x:v>12:40</x:v>
+      </x:c>
+      <x:c r="C10" s="114" t="str">
+        <x:v>화보 촬영 점심</x:v>
+      </x:c>
+      <x:c r="D10" s="116" t="n">
+        <x:v>135000</x:v>
+      </x:c>
+      <x:c r="E10" s="114" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F10" s="114" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G10" s="114" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H10" s="116" t="n">
+        <x:v>27000</x:v>
+      </x:c>
+      <x:c r="I10" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J10" s="114" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="44" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="B11" s="45" t="str">
+        <x:v>13:10</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>카메오 촬영 식사</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
+        <x:v>Seo, Manager Park</x:v>
+      </x:c>
+      <x:c r="F11" s="45" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H11" s="46" t="n">
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="I11" s="118" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J11" s="45" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="115" t="n">
         <x:v>46212</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B12" s="114" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C9" s="25" t="str">
+      <x:c r="C12" s="114" t="str">
         <x:v>안무 연습 일식</x:v>
       </x:c>
-      <x:c r="D9" s="34" t="n">
+      <x:c r="D12" s="116" t="n">
         <x:v>74000</x:v>
       </x:c>
-      <x:c r="E9" s="40" t="str">
+      <x:c r="E12" s="114" t="str">
         <x:v>Haru, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F9" s="40" t="str">
+      <x:c r="F12" s="114" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G9" s="28" t="n">
+      <x:c r="G12" s="114" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H9" s="37" t="n">
-        <x:f>ROUND(D9/G9,0)</x:f>
+      <x:c r="H12" s="116" t="n">
         <x:v>24667</x:v>
       </x:c>
-      <x:c r="I9" s="28" t="str">
-        <x:f>IF(H9&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I12" s="117" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J9" s="28" t="str">
+      <x:c r="J12" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="72" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B10" s="73" t="str">
-        <x:v>18:30</x:v>
-      </x:c>
-      <x:c r="C10" s="65" t="str">
-        <x:v>팬미팅 연습 저녁</x:v>
-      </x:c>
-      <x:c r="D10" s="80" t="n">
-        <x:v>145000</x:v>
-      </x:c>
-      <x:c r="E10" s="65" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="44" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>18:20</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>콘서트 리허설 저녁</x:v>
+      </x:c>
+      <x:c r="D13" s="46" t="n">
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="E13" s="45" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F10" s="73" t="str">
+      <x:c r="F13" s="45" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G10" s="76" t="n">
+      <x:c r="G13" s="45" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H10" s="77" t="n">
-        <x:f>ROUND(D10/G10,0)</x:f>
-        <x:v>29000</x:v>
-      </x:c>
-      <x:c r="I10" s="73" t="str">
-        <x:f>IF(H10&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="H13" s="46" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="I13" s="117" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J10" s="73" t="str">
+      <x:c r="J13" s="45" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="72" t="n">
-        <x:v>46215</x:v>
-      </x:c>
-      <x:c r="B11" s="73" t="str">
-        <x:v>12:10</x:v>
-      </x:c>
-      <x:c r="C11" s="65" t="str">
-        <x:v>콘텐츠 촬영 도시락</x:v>
-      </x:c>
-      <x:c r="D11" s="80" t="n">
-        <x:v>162000</x:v>
-      </x:c>
-      <x:c r="E11" s="65" t="str">
-        <x:v>Haru, Seo, Noa, Manager Park</x:v>
-      </x:c>
-      <x:c r="F11" s="73" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="115" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B14" s="114" t="str">
+        <x:v>13:00</x:v>
+      </x:c>
+      <x:c r="C14" s="114" t="str">
+        <x:v>월간회의 점심</x:v>
+      </x:c>
+      <x:c r="D14" s="116" t="n">
+        <x:v>138000</x:v>
+      </x:c>
+      <x:c r="E14" s="114" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F14" s="114" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G11" s="76" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H11" s="77" t="n">
-        <x:f>ROUND(D11/G11,0)</x:f>
-        <x:v>54000</x:v>
-      </x:c>
-      <x:c r="I11" s="73" t="str">
-        <x:v>승인 완료</x:v>
-      </x:c>
-      <x:c r="J11" s="73" t="str">
+      <x:c r="G14" s="114" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H14" s="116" t="n">
+        <x:v>27600</x:v>
+      </x:c>
+      <x:c r="I14" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J14" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="72" t="n">
-        <x:v>46216</x:v>
-      </x:c>
-      <x:c r="B12" s="73" t="str">
-        <x:v>13:00</x:v>
-      </x:c>
-      <x:c r="C12" s="65" t="str">
-        <x:v>월간회의 점심</x:v>
-      </x:c>
-      <x:c r="D12" s="80" t="n">
-        <x:v>138000</x:v>
-      </x:c>
-      <x:c r="E12" s="65" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="44" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>12:25</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>퍼포먼스 점검 점심</x:v>
+      </x:c>
+      <x:c r="D15" s="46" t="n">
+        <x:v>104000</x:v>
+      </x:c>
+      <x:c r="E15" s="45" t="str">
+        <x:v>Haru, Min, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F15" s="45" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H15" s="46" t="n">
+        <x:v>26000</x:v>
+      </x:c>
+      <x:c r="I15" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J15" s="45" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="115" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B16" s="114" t="str">
+        <x:v>18:20</x:v>
+      </x:c>
+      <x:c r="C16" s="114" t="str">
+        <x:v>마감 리허설 저녁</x:v>
+      </x:c>
+      <x:c r="D16" s="116" t="n">
+        <x:v>175000</x:v>
+      </x:c>
+      <x:c r="E16" s="114" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F12" s="73" t="str">
+      <x:c r="F16" s="114" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G12" s="76" t="n">
+      <x:c r="G16" s="114" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H12" s="77" t="n">
-        <x:f>ROUND(D12/G12,0)</x:f>
-        <x:v>27600</x:v>
-      </x:c>
-      <x:c r="I12" s="73" t="str">
-        <x:f>IF(H12&gt;$J$3,"승인 대기","자동 처리")</x:f>
-        <x:v>자동 처리</x:v>
-      </x:c>
-      <x:c r="J12" s="73" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="74" t="n">
-        <x:v>46218</x:v>
-      </x:c>
-      <x:c r="B13" s="75" t="str">
-        <x:v>18:20</x:v>
-      </x:c>
-      <x:c r="C13" s="69" t="str">
-        <x:v>마감 리허설 저녁</x:v>
-      </x:c>
-      <x:c r="D13" s="81" t="n">
-        <x:v>175000</x:v>
-      </x:c>
-      <x:c r="E13" s="69" t="str">
-        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
-      </x:c>
-      <x:c r="F13" s="75" t="str">
-        <x:v>Manager Park</x:v>
-      </x:c>
-      <x:c r="G13" s="78" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H13" s="79" t="n">
-        <x:f>ROUND(D13/G13,0)</x:f>
+      <x:c r="H16" s="116" t="n">
         <x:v>35000</x:v>
       </x:c>
-      <x:c r="I13" s="75" t="str">
-        <x:f>IF(H13&gt;$J$3,"승인 대기","자동 처리")</x:f>
+      <x:c r="I16" s="118" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J13" s="75" t="str">
+      <x:c r="J16" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1151,7 +1252,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94eed0a7b1964339"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22c3d3a39104ad2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1188,7 +1289,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-22 , 2026-07-21 동일 시간대 3건 승인 확인용 포함 , 앱 기본 식비에 자동 반영되지 않음</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-21 , 주 5일 평일 기준 , 2026-07-21 동일 시간대 3건 승인 확인용 포함</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1249,224 +1350,244 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="29" t="n">
+      <x:c r="A6" s="115" t="n">
         <x:v>46219</x:v>
       </x:c>
-      <x:c r="B6" s="26" t="str">
+      <x:c r="B6" s="114" t="str">
         <x:v>12:15</x:v>
       </x:c>
-      <x:c r="C6" s="23" t="str">
+      <x:c r="C6" s="114" t="str">
         <x:v>합주실 점심</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="n">
+      <x:c r="D6" s="116" t="n">
         <x:v>118000</x:v>
       </x:c>
-      <x:c r="E6" s="38" t="str">
+      <x:c r="E6" s="114" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F6" s="38" t="str">
+      <x:c r="F6" s="114" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G6" s="26" t="n">
+      <x:c r="G6" s="114" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="35" t="n">
+      <x:c r="H6" s="116" t="n">
         <x:v>29500</x:v>
       </x:c>
-      <x:c r="I6" s="110" t="str">
+      <x:c r="I6" s="117" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J6" s="26" t="str">
+      <x:c r="J6" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
-      <x:c r="A7" s="30" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="B7" s="27" t="str">
-        <x:v>11:40</x:v>
-      </x:c>
-      <x:c r="C7" s="24" t="str">
-        <x:v>방송국 도시락</x:v>
-      </x:c>
-      <x:c r="D7" s="33" t="n">
-        <x:v>132000</x:v>
-      </x:c>
-      <x:c r="E7" s="39" t="str">
+      <x:c r="A7" s="44" t="n">
+        <x:v>46220</x:v>
+      </x:c>
+      <x:c r="B7" s="45" t="str">
+        <x:v>18:10</x:v>
+      </x:c>
+      <x:c r="C7" s="45" t="str">
+        <x:v>쇼케이스 준비 저녁</x:v>
+      </x:c>
+      <x:c r="D7" s="46" t="n">
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="E7" s="45" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F7" s="39" t="str">
+      <x:c r="F7" s="45" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G7" s="27" t="n">
+      <x:c r="G7" s="45" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H7" s="36" t="n">
-        <x:v>33000</x:v>
-      </x:c>
-      <x:c r="I7" s="111" t="str">
+      <x:c r="H7" s="46" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="I7" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J7" s="45" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="32" customHeight="1">
+      <x:c r="A8" s="115" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="B8" s="114" t="str">
+        <x:v>12:20</x:v>
+      </x:c>
+      <x:c r="C8" s="114" t="str">
+        <x:v>광고 촬영 도시락</x:v>
+      </x:c>
+      <x:c r="D8" s="116" t="n">
+        <x:v>104000</x:v>
+      </x:c>
+      <x:c r="E8" s="114" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F8" s="114" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G8" s="114" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H8" s="116" t="n">
+        <x:v>26000</x:v>
+      </x:c>
+      <x:c r="I8" s="117" t="str">
+        <x:v>자동 처리</x:v>
+      </x:c>
+      <x:c r="J8" s="114" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="32" customHeight="1">
+      <x:c r="A9" s="44" t="n">
+        <x:v>46224</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>12:05</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>라디오 대기 식사</x:v>
+      </x:c>
+      <x:c r="D9" s="46" t="n">
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="str">
+        <x:v>Manager Choi</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H9" s="46" t="n">
+        <x:v>13500</x:v>
+      </x:c>
+      <x:c r="I9" s="118" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J7" s="27" t="str">
+      <x:c r="J9" s="45" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="30" t="n">
+    <x:row r="10">
+      <x:c r="A10" s="115" t="n">
         <x:v>46224</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
-        <x:v>12:05</x:v>
-      </x:c>
-      <x:c r="C8" s="24" t="str">
-        <x:v>라디오 대기 식사</x:v>
-      </x:c>
-      <x:c r="D8" s="33" t="n">
-        <x:v>54000</x:v>
-      </x:c>
-      <x:c r="E8" s="39" t="str">
+      <x:c r="B10" s="114" t="str">
+        <x:v>12:30</x:v>
+      </x:c>
+      <x:c r="C10" s="114" t="str">
+        <x:v>라디오 추가 음료</x:v>
+      </x:c>
+      <x:c r="D10" s="116" t="n">
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="E10" s="114" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F8" s="39" t="str">
+      <x:c r="F10" s="114" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="n">
+      <x:c r="G10" s="114" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H8" s="36" t="n">
-        <x:v>13500</x:v>
-      </x:c>
-      <x:c r="I8" s="111" t="str">
+      <x:c r="H10" s="116" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="I10" s="118" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J8" s="27" t="str">
+      <x:c r="J10" s="114" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="32" customHeight="1">
-      <x:c r="A9" s="31" t="n">
+    <x:row r="11">
+      <x:c r="A11" s="44" t="n">
         <x:v>46224</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
-        <x:v>12:30</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="str">
-        <x:v>라디오 추가 음료</x:v>
-      </x:c>
-      <x:c r="D9" s="34" t="n">
-        <x:v>24000</x:v>
-      </x:c>
-      <x:c r="E9" s="40" t="str">
+      <x:c r="B11" s="45" t="str">
+        <x:v>12:50</x:v>
+      </x:c>
+      <x:c r="C11" s="45" t="str">
+        <x:v>라디오 간식 결제</x:v>
+      </x:c>
+      <x:c r="D11" s="46" t="n">
+        <x:v>36000</x:v>
+      </x:c>
+      <x:c r="E11" s="45" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F9" s="40" t="str">
+      <x:c r="F11" s="45" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G9" s="28" t="n">
+      <x:c r="G11" s="45" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H9" s="37" t="n">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="I9" s="112" t="str">
+      <x:c r="H11" s="46" t="n">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="I11" s="118" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J9" s="28" t="str">
+      <x:c r="J11" s="45" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="72" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B10" s="73" t="str">
-        <x:v>12:50</x:v>
-      </x:c>
-      <x:c r="C10" s="65" t="str">
-        <x:v>라디오 간식 결제</x:v>
-      </x:c>
-      <x:c r="D10" s="80" t="n">
-        <x:v>36000</x:v>
-      </x:c>
-      <x:c r="E10" s="65" t="str">
-        <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
-      </x:c>
-      <x:c r="F10" s="73" t="str">
-        <x:v>Manager Choi</x:v>
-      </x:c>
-      <x:c r="G10" s="76" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H10" s="77" t="n">
-        <x:v>9000</x:v>
-      </x:c>
-      <x:c r="I10" s="113" t="str">
-        <x:v>승인 대기</x:v>
-      </x:c>
-      <x:c r="J10" s="73" t="str">
-        <x:v>인사 마스터</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="72"/>
-      <x:c r="B11" s="73"/>
-      <x:c r="C11" s="65"/>
-      <x:c r="D11" s="80"/>
-      <x:c r="E11" s="65"/>
-      <x:c r="F11" s="73"/>
-      <x:c r="G11" s="76"/>
-      <x:c r="H11" s="77"/>
-      <x:c r="I11" s="73"/>
-      <x:c r="J11" s="73"/>
-    </x:row>
     <x:row r="12">
-      <x:c r="A12" s="72"/>
-      <x:c r="B12" s="73"/>
-      <x:c r="C12" s="65"/>
-      <x:c r="D12" s="80"/>
-      <x:c r="E12" s="65"/>
-      <x:c r="F12" s="73"/>
-      <x:c r="G12" s="76"/>
-      <x:c r="H12" s="77"/>
-      <x:c r="I12" s="73"/>
-      <x:c r="J12" s="73"/>
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="74"/>
-      <x:c r="B13" s="75"/>
-      <x:c r="C13" s="69"/>
-      <x:c r="D13" s="81"/>
-      <x:c r="E13" s="69"/>
-      <x:c r="F13" s="75"/>
-      <x:c r="G13" s="78"/>
-      <x:c r="H13" s="79"/>
-      <x:c r="I13" s="75"/>
-      <x:c r="J13" s="75"/>
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="90"/>
-      <x:c r="B14" s="92"/>
-      <x:c r="C14" s="86"/>
-      <x:c r="D14" s="96"/>
-      <x:c r="E14" s="86"/>
-      <x:c r="F14" s="92"/>
-      <x:c r="G14" s="100"/>
-      <x:c r="H14" s="102"/>
-      <x:c r="I14" s="108"/>
-      <x:c r="J14" s="92"/>
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="91"/>
-      <x:c r="B15" s="93"/>
-      <x:c r="C15" s="87"/>
-      <x:c r="D15" s="97"/>
-      <x:c r="E15" s="87"/>
-      <x:c r="F15" s="93"/>
-      <x:c r="G15" s="101"/>
-      <x:c r="H15" s="103"/>
-      <x:c r="I15" s="109"/>
-      <x:c r="J15" s="93"/>
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1484,7 +1605,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd91234efe092456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2fef879247847de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add hourly approval samples for both groups
</commit_message>
<xml_diff>
--- a/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
+++ b/sample-data/식사 정보/Food-Fee_아이돌_식사_샘플데이터.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="R17a40d1aa3f642f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="R088776835ee740ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samildol 식사" sheetId="1" r:id="Re416aa694a914317"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="삼데헌 식사" sheetId="2" r:id="Rcbea2437c32e4601"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -141,8 +141,28 @@
         <x:fgColor rgb="FFFCE4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0E6F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="8">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -198,11 +218,25 @@
         <x:color rgb="FFE0A458"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="119">
+  <x:cellXfs count="129">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -460,6 +494,20 @@
     <x:xf numFmtId="200" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -832,7 +880,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 주 5일 평일 출퇴근 기록과 일정표에 연동 , 앱 기본 식비에 자동 반영되지 않음</x:v>
+        <x:v>정산 기간 2026-07-01 ~ 2026-07-15 , 2026-07-15 동일 시간대 3건 예외 승인 확인용 포함</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -852,6 +900,14 @@
         <x:v>30000</x:v>
       </x:c>
     </x:row>
+    <x:row r="4">
+      <x:c r="I4" s="122" t="str">
+        <x:v>동시간대 승인 기준</x:v>
+      </x:c>
+      <x:c r="J4" s="122" t="str">
+        <x:v>3건</x:v>
+      </x:c>
+    </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="18" t="str">
         <x:v>날짜</x:v>
@@ -885,34 +941,34 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="115" t="n">
+      <x:c r="A6" s="124" t="n">
         <x:v>46204</x:v>
       </x:c>
-      <x:c r="B6" s="114" t="str">
+      <x:c r="B6" s="123" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C6" s="114" t="str">
+      <x:c r="C6" s="123" t="str">
         <x:v>배민 연습실 식사</x:v>
       </x:c>
-      <x:c r="D6" s="116" t="n">
+      <x:c r="D6" s="125" t="n">
         <x:v>92000</x:v>
       </x:c>
-      <x:c r="E6" s="114" t="str">
+      <x:c r="E6" s="123" t="str">
         <x:v>Haru, Min, Seo, Lia, Manager Park</x:v>
       </x:c>
-      <x:c r="F6" s="114" t="str">
+      <x:c r="F6" s="123" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G6" s="114" t="n">
+      <x:c r="G6" s="123" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="116" t="n">
+      <x:c r="H6" s="125" t="n">
         <x:v>23000</x:v>
       </x:c>
-      <x:c r="I6" s="117" t="str">
+      <x:c r="I6" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J6" s="114" t="str">
+      <x:c r="J6" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -941,7 +997,7 @@
       <x:c r="H7" s="46" t="n">
         <x:v>25000</x:v>
       </x:c>
-      <x:c r="I7" s="117" t="str">
+      <x:c r="I7" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J7" s="45" t="str">
@@ -949,34 +1005,34 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="115" t="n">
+      <x:c r="A8" s="124" t="n">
         <x:v>46206</x:v>
       </x:c>
-      <x:c r="B8" s="114" t="str">
+      <x:c r="B8" s="123" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C8" s="114" t="str">
+      <x:c r="C8" s="123" t="str">
         <x:v>음악방송 도시락</x:v>
       </x:c>
-      <x:c r="D8" s="116" t="n">
+      <x:c r="D8" s="125" t="n">
         <x:v>165000</x:v>
       </x:c>
-      <x:c r="E8" s="114" t="str">
+      <x:c r="E8" s="123" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F8" s="114" t="str">
+      <x:c r="F8" s="123" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G8" s="114" t="n">
+      <x:c r="G8" s="123" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H8" s="116" t="n">
+      <x:c r="H8" s="125" t="n">
         <x:v>33000</x:v>
       </x:c>
-      <x:c r="I8" s="118" t="str">
+      <x:c r="I8" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J8" s="114" t="str">
+      <x:c r="J8" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1005,7 +1061,7 @@
       <x:c r="H9" s="46" t="n">
         <x:v>24000</x:v>
       </x:c>
-      <x:c r="I9" s="117" t="str">
+      <x:c r="I9" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J9" s="45" t="str">
@@ -1013,34 +1069,34 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="115" t="n">
+      <x:c r="A10" s="124" t="n">
         <x:v>46210</x:v>
       </x:c>
-      <x:c r="B10" s="114" t="str">
+      <x:c r="B10" s="123" t="str">
         <x:v>12:40</x:v>
       </x:c>
-      <x:c r="C10" s="114" t="str">
+      <x:c r="C10" s="123" t="str">
         <x:v>화보 촬영 점심</x:v>
       </x:c>
-      <x:c r="D10" s="116" t="n">
+      <x:c r="D10" s="125" t="n">
         <x:v>135000</x:v>
       </x:c>
-      <x:c r="E10" s="114" t="str">
+      <x:c r="E10" s="123" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F10" s="114" t="str">
+      <x:c r="F10" s="123" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G10" s="114" t="n">
+      <x:c r="G10" s="123" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H10" s="116" t="n">
+      <x:c r="H10" s="125" t="n">
         <x:v>27000</x:v>
       </x:c>
-      <x:c r="I10" s="117" t="str">
+      <x:c r="I10" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J10" s="114" t="str">
+      <x:c r="J10" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1069,7 +1125,7 @@
       <x:c r="H11" s="46" t="n">
         <x:v>42000</x:v>
       </x:c>
-      <x:c r="I11" s="118" t="str">
+      <x:c r="I11" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J11" s="45" t="str">
@@ -1077,34 +1133,34 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="115" t="n">
+      <x:c r="A12" s="124" t="n">
         <x:v>46212</x:v>
       </x:c>
-      <x:c r="B12" s="114" t="str">
+      <x:c r="B12" s="123" t="str">
         <x:v>12:00</x:v>
       </x:c>
-      <x:c r="C12" s="114" t="str">
+      <x:c r="C12" s="123" t="str">
         <x:v>안무 연습 일식</x:v>
       </x:c>
-      <x:c r="D12" s="116" t="n">
+      <x:c r="D12" s="125" t="n">
         <x:v>74000</x:v>
       </x:c>
-      <x:c r="E12" s="114" t="str">
+      <x:c r="E12" s="123" t="str">
         <x:v>Haru, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F12" s="114" t="str">
+      <x:c r="F12" s="123" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G12" s="114" t="n">
+      <x:c r="G12" s="123" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H12" s="116" t="n">
+      <x:c r="H12" s="125" t="n">
         <x:v>24667</x:v>
       </x:c>
-      <x:c r="I12" s="117" t="str">
+      <x:c r="I12" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J12" s="114" t="str">
+      <x:c r="J12" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1133,7 +1189,7 @@
       <x:c r="H13" s="46" t="n">
         <x:v>30000</x:v>
       </x:c>
-      <x:c r="I13" s="117" t="str">
+      <x:c r="I13" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J13" s="45" t="str">
@@ -1141,34 +1197,34 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="115" t="n">
+      <x:c r="A14" s="124" t="n">
         <x:v>46216</x:v>
       </x:c>
-      <x:c r="B14" s="114" t="str">
+      <x:c r="B14" s="123" t="str">
         <x:v>13:00</x:v>
       </x:c>
-      <x:c r="C14" s="114" t="str">
+      <x:c r="C14" s="123" t="str">
         <x:v>월간회의 점심</x:v>
       </x:c>
-      <x:c r="D14" s="116" t="n">
+      <x:c r="D14" s="125" t="n">
         <x:v>138000</x:v>
       </x:c>
-      <x:c r="E14" s="114" t="str">
+      <x:c r="E14" s="123" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F14" s="114" t="str">
+      <x:c r="F14" s="123" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G14" s="114" t="n">
+      <x:c r="G14" s="123" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H14" s="116" t="n">
+      <x:c r="H14" s="125" t="n">
         <x:v>27600</x:v>
       </x:c>
-      <x:c r="I14" s="117" t="str">
+      <x:c r="I14" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J14" s="114" t="str">
+      <x:c r="J14" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1197,7 +1253,7 @@
       <x:c r="H15" s="46" t="n">
         <x:v>26000</x:v>
       </x:c>
-      <x:c r="I15" s="117" t="str">
+      <x:c r="I15" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J15" s="45" t="str">
@@ -1205,34 +1261,130 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="115" t="n">
+      <x:c r="A16" s="124" t="n">
         <x:v>46218</x:v>
       </x:c>
-      <x:c r="B16" s="114" t="str">
+      <x:c r="B16" s="123" t="str">
+        <x:v>12:05</x:v>
+      </x:c>
+      <x:c r="C16" s="123" t="str">
+        <x:v>마감 리허설 점심</x:v>
+      </x:c>
+      <x:c r="D16" s="125" t="n">
+        <x:v>125000</x:v>
+      </x:c>
+      <x:c r="E16" s="123" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F16" s="123" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G16" s="123" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H16" s="125" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="I16" s="127" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J16" s="123" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="44" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>12:30</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>마감 리허설 추가 음료</x:v>
+      </x:c>
+      <x:c r="D17" s="46" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="E17" s="45" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F17" s="45" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H17" s="46" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I17" s="127" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="124" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B18" s="123" t="str">
+        <x:v>12:50</x:v>
+      </x:c>
+      <x:c r="C18" s="123" t="str">
+        <x:v>마감 리허설 간식 결제</x:v>
+      </x:c>
+      <x:c r="D18" s="125" t="n">
+        <x:v>35000</x:v>
+      </x:c>
+      <x:c r="E18" s="123" t="str">
+        <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
+      </x:c>
+      <x:c r="F18" s="123" t="str">
+        <x:v>Manager Park</x:v>
+      </x:c>
+      <x:c r="G18" s="123" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H18" s="125" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="I18" s="127" t="str">
+        <x:v>승인 대기</x:v>
+      </x:c>
+      <x:c r="J18" s="123" t="str">
+        <x:v>인사 마스터</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="44" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B19" s="45" t="str">
         <x:v>18:20</x:v>
       </x:c>
-      <x:c r="C16" s="114" t="str">
+      <x:c r="C19" s="45" t="str">
         <x:v>마감 리허설 저녁</x:v>
       </x:c>
-      <x:c r="D16" s="116" t="n">
+      <x:c r="D19" s="46" t="n">
         <x:v>175000</x:v>
       </x:c>
-      <x:c r="E16" s="114" t="str">
+      <x:c r="E19" s="45" t="str">
         <x:v>Haru, Min, Seo, Lia, Noa, Manager Park</x:v>
       </x:c>
-      <x:c r="F16" s="114" t="str">
+      <x:c r="F19" s="45" t="str">
         <x:v>Manager Park</x:v>
       </x:c>
-      <x:c r="G16" s="114" t="n">
+      <x:c r="G19" s="45" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H16" s="116" t="n">
+      <x:c r="H19" s="46" t="n">
         <x:v>35000</x:v>
       </x:c>
-      <x:c r="I16" s="118" t="str">
+      <x:c r="I19" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J16" s="114" t="str">
+      <x:c r="J19" s="45" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1252,7 +1404,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22c3d3a39104ad2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fd0917269294357"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1289,7 +1441,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>정산 기간 2026-07-16 ~ 2026-07-21 , 주 5일 평일 기준 , 2026-07-21 동일 시간대 3건 승인 확인용 포함</x:v>
+        <x:v>정산 기간 2026-07-16 ~ 2026-07-21 , 2026-07-21 동일 시간대 3건 예외 승인 확인용 포함</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1310,10 +1462,10 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="I4" s="85" t="str">
+      <x:c r="I4" s="122" t="str">
         <x:v>동시간대 승인 기준</x:v>
       </x:c>
-      <x:c r="J4" s="85" t="str">
+      <x:c r="J4" s="122" t="str">
         <x:v>3건</x:v>
       </x:c>
     </x:row>
@@ -1350,34 +1502,34 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="115" t="n">
+      <x:c r="A6" s="124" t="n">
         <x:v>46219</x:v>
       </x:c>
-      <x:c r="B6" s="114" t="str">
+      <x:c r="B6" s="123" t="str">
         <x:v>12:15</x:v>
       </x:c>
-      <x:c r="C6" s="114" t="str">
+      <x:c r="C6" s="123" t="str">
         <x:v>합주실 점심</x:v>
       </x:c>
-      <x:c r="D6" s="116" t="n">
+      <x:c r="D6" s="125" t="n">
         <x:v>118000</x:v>
       </x:c>
-      <x:c r="E6" s="114" t="str">
+      <x:c r="E6" s="123" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F6" s="114" t="str">
+      <x:c r="F6" s="123" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G6" s="114" t="n">
+      <x:c r="G6" s="123" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="116" t="n">
+      <x:c r="H6" s="125" t="n">
         <x:v>29500</x:v>
       </x:c>
-      <x:c r="I6" s="117" t="str">
+      <x:c r="I6" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J6" s="114" t="str">
+      <x:c r="J6" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1406,7 +1558,7 @@
       <x:c r="H7" s="46" t="n">
         <x:v>30000</x:v>
       </x:c>
-      <x:c r="I7" s="117" t="str">
+      <x:c r="I7" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
       <x:c r="J7" s="45" t="str">
@@ -1414,34 +1566,34 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="115" t="n">
+      <x:c r="A8" s="124" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="B8" s="114" t="str">
+      <x:c r="B8" s="123" t="str">
         <x:v>12:20</x:v>
       </x:c>
-      <x:c r="C8" s="114" t="str">
+      <x:c r="C8" s="123" t="str">
         <x:v>광고 촬영 도시락</x:v>
       </x:c>
-      <x:c r="D8" s="116" t="n">
+      <x:c r="D8" s="125" t="n">
         <x:v>104000</x:v>
       </x:c>
-      <x:c r="E8" s="114" t="str">
+      <x:c r="E8" s="123" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F8" s="114" t="str">
+      <x:c r="F8" s="123" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G8" s="114" t="n">
+      <x:c r="G8" s="123" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H8" s="116" t="n">
+      <x:c r="H8" s="125" t="n">
         <x:v>26000</x:v>
       </x:c>
-      <x:c r="I8" s="117" t="str">
+      <x:c r="I8" s="126" t="str">
         <x:v>자동 처리</x:v>
       </x:c>
-      <x:c r="J8" s="114" t="str">
+      <x:c r="J8" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1470,7 +1622,7 @@
       <x:c r="H9" s="46" t="n">
         <x:v>13500</x:v>
       </x:c>
-      <x:c r="I9" s="118" t="str">
+      <x:c r="I9" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J9" s="45" t="str">
@@ -1478,34 +1630,34 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="115" t="n">
+      <x:c r="A10" s="124" t="n">
         <x:v>46224</x:v>
       </x:c>
-      <x:c r="B10" s="114" t="str">
+      <x:c r="B10" s="123" t="str">
         <x:v>12:30</x:v>
       </x:c>
-      <x:c r="C10" s="114" t="str">
+      <x:c r="C10" s="123" t="str">
         <x:v>라디오 추가 음료</x:v>
       </x:c>
-      <x:c r="D10" s="116" t="n">
+      <x:c r="D10" s="125" t="n">
         <x:v>24000</x:v>
       </x:c>
-      <x:c r="E10" s="114" t="str">
+      <x:c r="E10" s="123" t="str">
         <x:v>원준석, 장현우, 김진현, 이준영, Manager Choi</x:v>
       </x:c>
-      <x:c r="F10" s="114" t="str">
+      <x:c r="F10" s="123" t="str">
         <x:v>Manager Choi</x:v>
       </x:c>
-      <x:c r="G10" s="114" t="n">
+      <x:c r="G10" s="123" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H10" s="116" t="n">
+      <x:c r="H10" s="125" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="I10" s="118" t="str">
+      <x:c r="I10" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
-      <x:c r="J10" s="114" t="str">
+      <x:c r="J10" s="123" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
     </x:row>
@@ -1534,7 +1686,7 @@
       <x:c r="H11" s="46" t="n">
         <x:v>9000</x:v>
       </x:c>
-      <x:c r="I11" s="118" t="str">
+      <x:c r="I11" s="127" t="str">
         <x:v>승인 대기</x:v>
       </x:c>
       <x:c r="J11" s="45" t="str">
@@ -1605,7 +1757,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2fef879247847de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcb5dbec48334266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>